<commit_message>
Publish course materials (e6bfabb0)
Generated by scripts/publish_student.py from the source repository at e6bfabb0: "W8: agent labs for both classes, old BERT material removed"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -542,7 +542,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,6 +553,12 @@
     <font>
       <sz val="14"/>
       <color rgb="FF1a3c6e"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -593,12 +599,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u/>
       <sz val="8"/>
       <color rgb="FF1a3c6e"/>
@@ -608,13 +608,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF7a7a7a"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="8"/>
-      <color rgb="FF1a3c6e"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -711,48 +704,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
@@ -764,37 +757,31 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="13" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1114,16 +1101,16 @@
   <dimension ref="A1:J34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="29" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="30" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="31" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="32" width="30.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="32" width="38.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="32" width="30.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="32" width="34.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="32" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="32" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="32" width="26.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="27" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="28" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="29" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="30" width="30.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="30" width="38.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="30" width="30.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="30" width="34.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="30" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="30" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="30" width="26.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="26">
@@ -1364,7 +1351,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="58" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="46.5" customFormat="1" s="5">
       <c r="A11" s="8">
         <v>5</v>
       </c>
@@ -1453,7 +1440,7 @@
       <c r="F14" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="15" t="s">
         <v>73</v>
       </c>
       <c r="H14" s="11"/>
@@ -1534,7 +1521,7 @@
       <c r="I17" s="11"/>
       <c r="J17" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="45">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="27">
       <c r="A18" s="13"/>
       <c r="B18" s="14"/>
       <c r="C18" s="10" t="s">
@@ -1549,7 +1536,7 @@
       <c r="F18" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="15" t="s">
         <v>92</v>
       </c>
       <c r="H18" s="11"/>
@@ -1608,7 +1595,7 @@
         <v>104</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="58" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33" customFormat="1" s="5">
       <c r="A21" s="8">
         <v>10</v>
       </c>
@@ -1632,7 +1619,7 @@
       <c r="I21" s="11"/>
       <c r="J21" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="84">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="35.25">
       <c r="A22" s="13"/>
       <c r="B22" s="14"/>
       <c r="C22" s="10" t="s">
@@ -1671,7 +1658,7 @@
         <v>53</v>
       </c>
       <c r="F23" s="11"/>
-      <c r="G23" s="21"/>
+      <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11" t="s">
         <v>115</v>
@@ -1693,7 +1680,7 @@
       <c r="F24" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="15" t="s">
         <v>120</v>
       </c>
       <c r="H24" s="11"/>
@@ -1747,7 +1734,7 @@
         <v>132</v>
       </c>
       <c r="F26" s="11"/>
-      <c r="G26" s="21"/>
+      <c r="G26" s="11"/>
       <c r="H26" s="11" t="s">
         <v>133</v>
       </c>
@@ -1775,7 +1762,7 @@
       </c>
       <c r="G27" s="11"/>
       <c r="H27" s="11"/>
-      <c r="I27" s="22" t="s">
+      <c r="I27" s="20" t="s">
         <v>139</v>
       </c>
       <c r="J27" s="11"/>
@@ -1793,7 +1780,7 @@
         <v>20</v>
       </c>
       <c r="F28" s="11"/>
-      <c r="G28" s="21"/>
+      <c r="G28" s="11"/>
       <c r="H28" s="11"/>
       <c r="I28" s="11" t="s">
         <v>141</v>
@@ -1803,8 +1790,8 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="24" customFormat="1" s="5">
-      <c r="A29" s="23"/>
-      <c r="B29" s="24" t="s">
+      <c r="A29" s="21"/>
+      <c r="B29" s="22" t="s">
         <v>143</v>
       </c>
       <c r="C29" s="16" t="s">
@@ -1855,7 +1842,7 @@
       <c r="F31" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="G31" s="20" t="s">
+      <c r="G31" s="15" t="s">
         <v>151</v>
       </c>
       <c r="H31" s="11" t="s">
@@ -1879,7 +1866,7 @@
         <v>155</v>
       </c>
       <c r="F32" s="11"/>
-      <c r="G32" s="21"/>
+      <c r="G32" s="11"/>
       <c r="H32" s="11"/>
       <c r="I32" s="11" t="s">
         <v>156</v>
@@ -1887,7 +1874,7 @@
       <c r="J32" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="58" customFormat="1" s="5">
-      <c r="A33" s="25">
+      <c r="A33" s="23">
         <v>15</v>
       </c>
       <c r="B33" s="18" t="s">
@@ -1903,7 +1890,7 @@
         <v>159</v>
       </c>
       <c r="F33" s="11"/>
-      <c r="G33" s="21"/>
+      <c r="G33" s="11"/>
       <c r="H33" s="11"/>
       <c r="I33" s="11" t="s">
         <v>160</v>
@@ -1913,30 +1900,30 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="64" customFormat="1" s="5">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="D34" s="28" t="s">
+      <c r="D34" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="E34" s="28" t="s">
+      <c r="E34" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="F34" s="28"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="28" t="s">
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="I34" s="28" t="s">
+      <c r="I34" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="J34" s="28" t="s">
+      <c r="J34" s="26" t="s">
         <v>169</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish course materials (0c137903)
Generated by scripts/publish_student.py from the source repository at 0c137903: "W9: decoding walkthrough instructor lab and student lab, new Quiz 5, remove stale W9 content"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -420,7 +420,7 @@
     <t>Wed Nov 11</t>
   </si>
   <si>
-    <t>Agentic workflows: chaining, routing, parallelization, multi-agent, reflection and evaluator-optimizer, and when NOT to use an agent</t>
+    <t>Agentic Workflows &amp; Midterm Review</t>
   </si>
   <si>
     <t>Lecture, Whiteboard, Discussion</t>
@@ -542,7 +542,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -558,7 +558,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -582,12 +582,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -736,52 +730,52 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="12" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="11" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="10" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="7" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1159,7 +1153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="58" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="46.5" customFormat="1" s="5">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1187,7 +1181,7 @@
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="70">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="46.5">
       <c r="A4" s="13"/>
       <c r="B4" s="14"/>
       <c r="C4" s="10" t="s">
@@ -1211,7 +1205,7 @@
       </c>
       <c r="J4" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="70" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="46.5" customFormat="1" s="5">
       <c r="A5" s="8">
         <v>2</v>
       </c>

</xml_diff>